<commit_message>
AI audit log third time
</commit_message>
<xml_diff>
--- a/14_05_2026___dbfd2274ec8368baecac0ed92ccb5583...xlsx
+++ b/14_05_2026___dbfd2274ec8368baecac0ed92ccb5583...xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\wdp301-aiauditlog-php2422005\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -929,58 +929,163 @@
     <t>Research stage</t>
   </si>
   <si>
-    <t>Phản hồi: AI so sánh chi tiết và đưa ra kết luận nên dùng JWT vì xu hướng hiện nay là REST API stateless, phù hợp nếu FE tách rời BE.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI gợi ý Chart.js, Chartist.js và một thư viện tên là "TinyChartJS".</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI gợi ý 2 cách: (1) Tạo 1 bảng User có cột RoleID, (2) Tạo 3 bảng User, Admin, Seller riêng biệt.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI nói với 500 items thì có thể fetch hết về FE lọc cho mượt (O(n)), đỡ tốn query database liên tục.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI xác nhận đúng, giải thích rằng Regex này bắt buộc 8 ký tự, có ít nhất 1 chữ cái và 1 chữ số.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI xác nhận code đúng và chỉ ra vài edge cases như page nhỏ hơn 1 hoặc lớn hơn tổng số page.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: AI chỉ ra edge case đúng nhưng bỏ sót việc tính toán tổng số page bị sai nếu total items chia hết cho items_per_page.
+    <t xml:space="preserve">Abstraction
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi đang nghiên cứu cách cào dữ liệu (Crawlee) từ trang Winmart. HTML của họ chứa quá nhiều thẻ lồng nhau và thay đổi liên tục. Theo nguyên lý Abstraction, thay vì viết DOM Parser phức tạp (Cheerio), tôi có thể lấy toàn bộ Raw Text của trang và dùng AI LLM (Gemini) để tự động trích xuất Tên, SKU, Giá được không? Phân tích ưu nhược điểm của cách này." 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tôi cần thiết kế tính năng 'AI Gợi ý giá hàng loạt' cho danh sách sản phẩm đối thủ. Nếu gửi toàn bộ mảng data cùng lúc sẽ bị lỗi Rate Limit của API. Hãy phân rã (decompose) bài toán này thành các module xử lý nhỏ hơn: cách UI hiển thị trạng thái đang xử lý, và cách Backend hoặc Frontend kiểm soát hàng đợi (queue) để gọi API an toàn." 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pattern Recognition
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Trong hệ thống Admin, tôi nhận thấy một mẫu (pattern) lỗi UX lặp lại ở trang Quản lý Banner và Kho hàng: hàm window.confirm() hiển thị popup 'localhost says...' mặc định rất thiếu chuyên nghiệp. Tôi muốn thay thế bằng Custom Modal. Hãy phân tích những State cốt lõi nào cần phải có để tái tạo lại luồng 'chặn - chờ xác nhận - thực thi' này trong React?" 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algorithm
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Thuật toán 'Xóa nhiều sản phẩm' của tôi đang gặp lỗi. Logic hiện tại: Lọc các _id được check -&gt; gom thành mảng idsToDelete -&gt; gửi POST request qua Axios. Dù xóa 1 sản phẩm thành công, nhưng xóa nhiều thì báo 'Có lỗi xảy ra'. Hãy liệt kê các điểm mù (blind spots) trong cơ chế truyền mảng JSON qua Axios và cách Mongoose $in cast ObjectId để tôi tự trace lỗi." 
+</t>
+  </si>
+  <si>
+    <t>AI so sánh chi tiết và đưa ra kết luận nên dùng JWT vì xu hướng hiện nay là REST API stateless, phù hợp nếu FE tách rời BE.</t>
+  </si>
+  <si>
+    <t>AI gợi ý Chart.js, Chartist.js và một thư viện tên là "TinyChartJS".</t>
+  </si>
+  <si>
+    <t>AI gợi ý 2 cách: (1) Tạo 1 bảng User có cột RoleID, (2) Tạo 3 bảng User, Admin, Seller riêng biệt.</t>
+  </si>
+  <si>
+    <t>AI nói với 500 items thì có thể fetch hết về FE lọc cho mượt (O(n)), đỡ tốn query database liên tục.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> AI xác nhận đúng, giải thích rằng Regex này bắt buộc 8 ký tự, có ít nhất 1 chữ cái và 1 chữ số.</t>
+  </si>
+  <si>
+    <t>AI xác nhận code đúng và chỉ ra vài edge cases như page nhỏ hơn 1 hoặc lớn hơn tổng số page.</t>
+  </si>
+  <si>
+    <t>AI khuyên đúng xu hướng, nhưng JWT có nhược điểm bảo mật là khó thu hồi (revoke) ngay lập tức khi user nhấn logout.
+Contextualization: Project có FE và BE tách biệt, dùng fetch API. JWT dễ setup hơn config Cookie CORS đa miền.
+Creative Synthesis: Đồng ý dùng JWT nhưng quyết định set thời gian sống (expiration) của token rất ngắn (15 phút) để tăng tính an toàn.
+Decision Ownership: Chốt sử dụng JWT Auth Token lưu ở localStorage để dev nhanh, bù đắp yếu điểm security bằng short-lived access token.</t>
+  </si>
+  <si>
+    <t>AI đưa ra "TinyChartJS" nghe rất hợp lý vì yêu cầu "nhẹ". Nhưng cần xác minh lại độ uy tín.
+Contextualization: Dùng thư viện lạ có nguy cơ không có document, lúc có bug sẽ không fix kịp trước hạn nộp project.
+Creative Synthesis: Tìm tên "TinyChartJS" trên Github và NPM thì phát hiện ra nó rất ít sao và ngừng maintain (Hallucination/Outdated Info).
+Decision Ownership: Loại bỏ thư viện AI xui, chốt sử dụng Chart.js vì có document cực kỳ rõ ràng, nhiều support trên StackOverflow.</t>
+  </si>
+  <si>
+    <t>Cách 2 (3 bảng riêng) của AI quá cồng kềnh, bị lặp lại các cột chung như Email, Password.
+Contextualization: Website hiện tại chủ yếu là 2 role Admin/Customer, các dữ liệu cá nhân là như nhau.
+Creative Synthesis: Tôi chọn cách 1 nhưng thay vì làm hẳn bảng Role riêng biệt (cần JOIN), tôi dùng kiểu ENUM ('ADMIN', 'CUSTOMER') trong bảng User.
+Decision Ownership: Áp dụng thiết kế 1 bảng User với cột ENUM. Đơn giản hóa kiến trúc DB cho phù hợp với quy mô project thay vì làm quá rườm rà như AI khuyên.</t>
+  </si>
+  <si>
+    <t>Lọc FE nhanh thật, nhưng nếu mỗi sản phẩm có ảnh nặng và text dài, fetch 500 cái cùng lúc sẽ làm sập băng thông.
+Contextualization: Mục tiêu là First Contentful Paint phải &lt; 3s. Tải cục data bự sẽ vi phạm tiêu chuẩn tối ưu.
+Creative Synthesis: Bác bỏ hoàn toàn gợi ý của AI. Chuyển logic xuống BE, dùng Query params (?price_min=100) và câu lệnh SQL WHERE.
+Decision Ownership: Quyết định thực hiện Filtering và Pagination ở Backend để đảm bảo trang load nhanh, tuân thủ best practice.</t>
+  </si>
+  <si>
+    <t>AI giải thích chức năng cơ bản đúng, nhưng Regex này KHÔNG cho phép gõ ký tự đặc biệt (!@#$). Nếu nhập vào sẽ báo lỗi.
+Contextualization: Form đăng ký của nhóm yêu cầu mật khẩu bảo mật cao (phải có ký tự đặc biệt) để chấm điểm cộng.
+Creative Synthesis: Đem test trên Regex101 và xác nhận lỗi thiếu special chars. Tôi tự update Regex thành có đủ chữ hoa, thường, số, ký tự đặc biệt.
+Decision Ownership: Không tin tưởng 100% code do AI sinh. Quyết định tự mod lại Regex phức tạp hơn để đảm bảo tính năng hoạt động chuẩn xác.</t>
+  </si>
+  <si>
+    <t>AI chỉ ra edge case đúng nhưng bỏ sót việc tính toán tổng số page bị sai nếu total items chia hết cho items_per_page.
 Contextualization: API trả về số lượng động. Nếu items_per_page = 10, total=10 thì thuật toán của AI lại tính ra 2 page thay vì 1.
 Creative Synthesis: Tôi test tay bằng Console và phát hiện lỗi math. Tôi sửa lại công thức thành Math.ceil(totalItems / itemsPerPage).
 Decision Ownership: Tự viết lại hàm tính page dùng Math.ceil thay vì if/else cồng kềnh của AI, giúp code an toàn và tránh bug.</t>
   </si>
   <si>
-    <t>Critical Thinking: AI khuyên đúng xu hướng, nhưng JWT có nhược điểm bảo mật là khó thu hồi (revoke) ngay lập tức khi user nhấn logout.
-Contextualization: Project có FE và BE tách biệt, dùng fetch API. JWT dễ setup hơn config Cookie CORS đa miền.
-Creative Synthesis: Đồng ý dùng JWT nhưng quyết định set thời gian sống (expiration) của token rất ngắn (15 phút) để tăng tính an toàn.
-Decision Ownership: Chốt sử dụng JWT Auth Token lưu ở localStorage để dev nhanh, bù đắp yếu điểm security bằng short-lived access token.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: AI đưa ra "TinyChartJS" nghe rất hợp lý vì yêu cầu "nhẹ". Nhưng cần xác minh lại độ uy tín.
-Contextualization: Dùng thư viện lạ có nguy cơ không có document, lúc có bug sẽ không fix kịp trước hạn nộp project.
-Creative Synthesis: Tìm tên "TinyChartJS" trên Github và NPM thì phát hiện ra nó rất ít sao và ngừng maintain (Hallucination/Outdated Info).
-Decision Ownership: Loại bỏ thư viện AI xui, chốt sử dụng Chart.js vì có document cực kỳ rõ ràng, nhiều support trên StackOverflow.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Cách 2 (3 bảng riêng) của AI quá cồng kềnh, bị lặp lại các cột chung như Email, Password.
-Contextualization: Website hiện tại chủ yếu là 2 role Admin/Customer, các dữ liệu cá nhân là như nhau.
-Creative Synthesis: Tôi chọn cách 1 nhưng thay vì làm hẳn bảng Role riêng biệt (cần JOIN), tôi dùng kiểu ENUM ('ADMIN', 'CUSTOMER') trong bảng User.
-Decision Ownership: Áp dụng thiết kế 1 bảng User với cột ENUM. Đơn giản hóa kiến trúc DB cho phù hợp với quy mô project thay vì làm quá rườm rà như AI khuyên.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: Lọc FE nhanh thật, nhưng nếu mỗi sản phẩm có ảnh nặng và text dài, fetch 500 cái cùng lúc sẽ làm sập băng thông.
-Contextualization: Mục tiêu là First Contentful Paint phải &lt; 3s. Tải cục data bự sẽ vi phạm tiêu chuẩn tối ưu.
-Creative Synthesis: Bác bỏ hoàn toàn gợi ý của AI. Chuyển logic xuống BE, dùng Query params (?price_min=100) và câu lệnh SQL WHERE.
-Decision Ownership: Quyết định thực hiện Filtering và Pagination ở Backend để đảm bảo trang load nhanh, tuân thủ best practice.</t>
-  </si>
-  <si>
-    <t>Critical Thinking: AI giải thích chức năng cơ bản đúng, nhưng Regex này KHÔNG cho phép gõ ký tự đặc biệt (!@#$). Nếu nhập vào sẽ báo lỗi.
-Contextualization: Form đăng ký của nhóm yêu cầu mật khẩu bảo mật cao (phải có ký tự đặc biệt) để chấm điểm cộng.
-Creative Synthesis: Đem test trên Regex101 và xác nhận lỗi thiếu special chars. Tôi tự update Regex thành có đủ chữ hoa, thường, số, ký tự đặc biệt.
-Decision Ownership: Không tin tưởng 100% code do AI sinh. Quyết định tự mod lại Regex phức tạp hơn để đảm bảo tính năng hoạt động chuẩn xác.</t>
+    <t xml:space="preserve">AI đồng tình và đưa ra so sánh: DOM Parser nhanh, rẻ nhưng dễ gãy (brittle) khi web thay đổi UI. Dùng LLM linh hoạt, chịu lỗi tốt (fault-tolerant) nhưng chậm và tốn chi phí gọi API. AI cũng cung cấp đoạn prompt mẫu để gửi Raw Text cho LLM. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất chia làm 3 phần: 1) Nút trigger trên UI đổi trạng thái (Loading spinner). 2) Hàm chạy vòng lặp tuần tự (For...of) trên danh sách các ID được chọn thay vì Promise.all. 3) Trả kết quả từng bước (hoặc gom lại) để update state bulkSuggestResults. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI phân tích và đưa ra 3 State cốt lõi cần quản lý: isOpen (boolean để đóng/mở), targetId (lưu ID của item chuẩn bị thao tác), và isLoading (hiệu ứng loading khi chờ API xử lý). 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI liệt kê 3 điểm mù: 1) Request gửi đi dạng { ids: [...] } có thể bị Express hiểu sai nếu thiếu body-parser. 2) Mảng có chứa giá trị undefined/null gây lỗi CastError của Mongoose. 3) Catch block ở Frontend đang nuốt lỗi (Swallow errors) khiến thông báo bị chung chung. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tôi nhận thấy tính ổn định của hệ thống quan trọng hơn tốc độ cào (do cào chạy ngầm). Tôi quyết định lược bỏ việc bóc tách HTML phức tạp (Abstraction), chỉ lấy innerText của thẻ body và gọi API Gemini để parse dữ liệu. Để khắc phục nhược điểm về tốc độ và chi phí (Rate Limit) mà AI cảnh báo, tôi chủ động thêm hàm setTimeout(12000) để delay giữa các request.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất dùng vòng lặp tuần tự là chính xác để tránh Rate Limit. Tuy nhiên, thay vì nhồi nhét toàn bộ logic gọi API vào file ManageInventoryPage.tsx như code mẫu của AI (gây phình to component), tôi quyết định tự phân rã thêm: tách hẳn logic gọi AI sang một file service riêng (ai.service.ts), UI chỉ chịu trách nhiệm lặp, hiển thị trạng thái &lt;RefreshCw className="animate-spin"/&gt; và chờ kết quả.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phân tích của AI về các State là rất chuẩn xác (Pattern Recognition). Tôi đã áp dụng để tạo Custom Modal. Tuy nhiên, khi kiểm thử luồng "Xóa nhiều" (Bulk Delete), tôi phát hiện AI chưa xử lý trường hợp ID truyền vào là một Mảng (Array) thay vì String. Tôi đã tự suy luận, điều chỉnh lại logic, bổ sung biến cờ crawledIsBulkDelete để phân biệt và chọn đúng ID(s) (idsToDelete) từ mảng đã chọn hoặc ID đơn lẻ truyền xuống API.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dựa trên gợi ý (3) của AI về việc "nuốt lỗi", tôi nhận ra mình không thể debug vì thông báo lỗi đã bị ghi đè thành câu tĩnh "Có lỗi xảy ra khi xóa". Quyết định của tôi: Tạm thời thay thế code hiển thị lỗi thành `err.response?.data?.message
+</t>
+  </si>
+  <si>
+    <t>Decomposition / Process</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Làm sao để tích hợp bộ cào dữ liệu Playwright vào Backend chạy ngầm mỗi 2h sáng, nhưng vẫn có nút bật/tắt thủ công ở giao diện Quản lý Kho? Khi bật phải vô hiệu hóa các nút Sửa/Xóa." 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI cung cấp cấu trúc Cron job bên BE (node-cron) và code UI bên FE, kèm API /api/crawler/start và /stop. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tôi nhận thấy AI xử lý việc disable nút khá thủ công. Tôi quyết định yêu cầu AI giữ nguyên style của nút "Thêm sản phẩm mới" để đảm bảo UI nhất quán, đồng thời tự bổ sung thêm cơ chế Polling (gọi API /status liên tục) để Frontend luôn đồng bộ chính xác trạng thái với Backend dù người dùng có F5 lại trang (Abstracting UI state).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluation
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Sau khi đổi logic nhận diện URL, hệ thống báo lỗi 404 với gemini-1.5-flash. Khi đổi sang gemini-2.5-flash lại báo limit: 20 (hết hạn ngạch). Có giải pháp nào khác không?" 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI cho biết model 1.5 đã bị loại bỏ, và tự động chuyển sang model gemini-2.0-flash-lite để mong tìm kiếm gói miễn phí. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI loay hoay thay đổi cấu hình mã model (2.0-flash-lite) nhưng vẫn trả về limit: 0 (Google khóa hoàn toàn gói free).
+Tôi nhận định không thể phụ thuộc vào việc "vá víu code" nếu bản chất vấn đề nằm ở chính sách Infrastructure của Google. Tôi quyết định khôi phục lại code về model ổn định nhất (gemini-2.5-flash), ngừng yêu cầu AI sửa code, và giải quyết triệt để bằng cách tạo một API Key mới tinh từ tài khoản Gmail khác để Reset hạn ngạch.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Tại sao khi chạy crawler lại liên tục báo lỗi 'AI Parsing Error: 429 Quota exceeded'? Dưới đây là log:
+INFO: Processing https://winmart.vn/gia-sieu-re--c114"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI phân tích lỗi 429 là do quá giới hạn API Gemini (15 req/phút). Đề xuất giảm maxConcurrency xuống 1 và thêm setTimeout(4500). </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất giải pháp giảm tốc độ cào rất cơ bản (rate-limiting). Dù đã ép trễ 4.5s, lỗi vẫn xảy ra. Đọc lại log, tôi nhận ra một Pattern (Mẫu): Crawler đang vơ vét cả các trang danh mục (có đuôi --c) thay vì chỉ trang sản phẩm (đuôi --s). AI ban đầu viết điều kiện nhận diện sai: "Chỉ cần có nút 'Thêm vào giỏ' là trang sản phẩm" (Oversimplification).
+Tôi đã phân tích lại cấu trúc URL của Winmart và tự chỉ đạo AI viết lại logic bằng Regex chỉ bắt các link có đuôi --s\d+.
+</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1060,7 +1165,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1395,7 +1506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.8984375" customWidth="1"/>
@@ -1517,7 +1628,7 @@
       <c r="D7" s="6"/>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1528,13 +1639,13 @@
         <v>24</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="7" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E8" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1545,13 +1656,13 @@
         <v>25</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="7" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="124.2" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1562,13 +1673,13 @@
         <v>26</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E10" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1579,13 +1690,13 @@
         <v>27</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E11" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1596,13 +1707,13 @@
         <v>28</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E12" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1613,10 +1724,129 @@
         <v>29</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="96.6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="110.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="69" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>38</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="110.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="96.6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>